<commit_message>
feat: Add KHM to CAMBODIA mapping for origin country processing.
</commit_message>
<xml_diff>
--- a/data/law_label_data.xlsx
+++ b/data/law_label_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/planet.cat/Documents/jy_code_workspace/label_generator/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{231B490A-DFF6-F14E-BC08-C9A526998ED1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B99DE9E-565A-4D4D-B67E-0737246B17BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="35">
   <si>
     <t>default_code</t>
   </si>
@@ -280,9 +280,6 @@
   </si>
   <si>
     <t>PER. No</t>
-  </si>
-  <si>
-    <t>Origin (CN/VN)</t>
   </si>
   <si>
     <t>UT 70028(CN)</t>
@@ -417,6 +414,14 @@
       </rPr>
       <t>100% POLYESTER FIBER</t>
     </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Origin (CN/VN/KHM)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>KHM</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -918,10 +923,10 @@
         <v>18</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>19</v>
+        <v>33</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="230.5" customHeight="1">
@@ -929,16 +934,16 @@
         <v>3</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>17</v>
       </c>
       <c r="D2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F2" t="s">
         <v>30</v>
@@ -955,13 +960,13 @@
         <v>17</v>
       </c>
       <c r="D3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F3" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="169.5" customHeight="1">
@@ -972,13 +977,13 @@
         <v>7</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="169.5" customHeight="1">
@@ -989,13 +994,13 @@
         <v>9</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F5" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="169.5" customHeight="1">
@@ -1006,13 +1011,13 @@
         <v>11</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="169.5" customHeight="1">
@@ -1020,19 +1025,19 @@
         <v>12</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="169.5" customHeight="1">
@@ -1043,13 +1048,13 @@
         <v>14</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E8" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="169.5" customHeight="1">
@@ -1060,17 +1065,25 @@
         <v>16</v>
       </c>
       <c r="C9" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E9" t="s">
+        <v>21</v>
+      </c>
+      <c r="F9" t="s">
         <v>29</v>
-      </c>
-      <c r="E9" t="s">
-        <v>22</v>
-      </c>
-      <c r="F9" t="s">
-        <v>30</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
+  <dataValidations count="2">
+    <dataValidation type="list" imeMode="off" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F1:F1048576" xr:uid="{A7A594BB-3937-FA4A-84CC-7EE2D273797F}">
+      <formula1>"CN, VN, KHM"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E1:E1048576" xr:uid="{F312475C-390A-5143-85D6-61D8E4B0F0B1}">
+      <formula1>"Mopio,Castlery"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: generate label 19
</commit_message>
<xml_diff>
--- a/data/law_label_data.xlsx
+++ b/data/law_label_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/planet.cat/Documents/jy_code_workspace/label_generator/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B99DE9E-565A-4D4D-B67E-0737246B17BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7134D60A-257E-2846-919A-DCCF3B31C518}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
         <b/>
         <sz val="12"/>
         <color rgb="FFFF0000"/>
-        <rFont val="等线"/>
+        <rFont val="Calibri"/>
         <family val="3"/>
         <charset val="134"/>
         <scheme val="minor"/>
@@ -56,7 +56,7 @@
         <b/>
         <sz val="12"/>
         <color theme="1"/>
-        <rFont val="等线"/>
+        <rFont val="Calibri"/>
         <family val="3"/>
         <charset val="134"/>
         <scheme val="minor"/>
@@ -223,55 +223,7 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">
-BODY
-95% POLYURETHANE FOAM PAD 
-5% POLYESTER FIBER BATTING
-SEAT CUSHION (1):
-90% POLYURETHANE FOAM PAD 
-10% POLYESTER FIBER BATTING
-COIL POCKET SPRING  
-BACK CUSHION  (1):
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>100% POLYESTER FIBER</t>
-    </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>EC2005 Modular Storage 2 Seater</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">
-BODY
-95% POLYURETHANE FOAM PAD 
-5% POLYESTER FIBER BATTING
-SEAT CUSHION (1):
-90% POLYURETHANE FOAM PAD 
-10% POLYESTER FIBER BATTING
-COIL POCKET SPRING  
-BACK CUSHION  (2):
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>100% POLYESTER FIBER</t>
-    </r>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -366,6 +318,14 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
+    <t>Origin (CN/VN/KHM)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>KHM</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
     <r>
       <rPr>
         <sz val="10"/>
@@ -414,15 +374,52 @@
       </rPr>
       <t>100% POLYESTER FIBER</t>
     </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Origin (CN/VN/KHM)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>KHM</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">
+BODY
+95% POLYURETHANE FOAM PAD 
+5% POLYESTER FIBER BATTING
+SEAT CUSHION (1):
+90% POLYURETHANE FOAM PAD 
+10% POLYESTER FIBER BATTING
+COIL POCKET SPRING  
+BACK CUSHION  (1):
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>100% POLYESTER FIBER</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">
+BBDY
+95% POLYURETHANE FOAM PAD 
+5% POLYESTER FIBER BATTING
+SEAT CUSHION (1):
+90% POLYURETHANE FOAM PAD 
+10% POLYESTER FIBER BATTING
+COIL POCKET SPRING  
+BACK CUSHION  (2):
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>100% POLYESTER FIBER</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -433,13 +430,13 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -447,7 +444,7 @@
     <font>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -456,7 +453,7 @@
       <b/>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -465,7 +462,7 @@
       <b/>
       <sz val="12"/>
       <color rgb="FFFF0000"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -514,7 +511,7 @@
       <b/>
       <sz val="12"/>
       <color rgb="FF000000"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="4"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -621,7 +618,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="常规 3" xfId="1" xr:uid="{ABE23CD4-8A8F-4323-AF65-D6D4E5A327EE}"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -920,13 +917,13 @@
         <v>2</v>
       </c>
       <c r="D1" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="E1" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="E1" s="10" t="s">
-        <v>20</v>
-      </c>
       <c r="F1" s="10" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="230.5" customHeight="1">
@@ -937,16 +934,16 @@
         <v>32</v>
       </c>
       <c r="C2" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" t="s">
         <v>17</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>19</v>
       </c>
-      <c r="E2" t="s">
-        <v>21</v>
-      </c>
       <c r="F2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="169.5" customHeight="1">
@@ -957,16 +954,16 @@
         <v>5</v>
       </c>
       <c r="C3" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" t="s">
         <v>17</v>
       </c>
-      <c r="D3" t="s">
-        <v>19</v>
-      </c>
       <c r="E3" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F3" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="169.5" customHeight="1">
@@ -977,13 +974,13 @@
         <v>7</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E4" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="169.5" customHeight="1">
@@ -994,13 +991,13 @@
         <v>9</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E5" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F5" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="169.5" customHeight="1">
@@ -1011,13 +1008,13 @@
         <v>11</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="E6" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F6" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="169.5" customHeight="1">
@@ -1025,19 +1022,19 @@
         <v>12</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D7" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E7" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F7" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="169.5" customHeight="1">
@@ -1045,33 +1042,33 @@
         <v>13</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>14</v>
+        <v>33</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E8" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F8" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="169.5" customHeight="1">
       <c r="A9" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>16</v>
+        <v>34</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E9" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F9" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Add 'IRON PAD' to term configuration, remove devcontainer setup, and update gitignore to exclude `law_label_data.xlsx`.
</commit_message>
<xml_diff>
--- a/data/law_label_data.xlsx
+++ b/data/law_label_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/planet.cat/Documents/jy_code_workspace/label_generator/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7134D60A-257E-2846-919A-DCCF3B31C518}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E94D6F85-9613-E440-9EA1-82FA65EA6685}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -401,11 +401,11 @@
   <si>
     <r>
       <t xml:space="preserve">
-BBDY
+BODY
 95% POLYURETHANE FOAM PAD 
 5% POLYESTER FIBER BATTING
 SEAT CUSHION (1):
-90% POLYURETHANE FOAM PAD 
+90% FELT
 10% POLYESTER FIBER BATTING
 COIL POCKET SPRING  
 BACK CUSHION  (2):

</xml_diff>